<commit_message>
Add project organization to directory
</commit_message>
<xml_diff>
--- a/4_General_Resources/SpeciesCode.xlsx
+++ b/4_General_Resources/SpeciesCode.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanco\Desktop\ResearchR\Final_Bio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanco\Desktop\ResearchR\Uncertainty_2025\4_General_Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B1E84F-6B26-4717-AAFE-D8298E1AC2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79471CDF-3E12-4D66-9C3B-BAFD67CBB05F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -468,38 +468,6 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -594,13 +562,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -610,6 +571,45 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -626,14 +626,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{324706FF-7CD4-4822-824E-9DCAB8D4079B}" name="Table1" displayName="Table1" ref="A1:F38" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="7" tableBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{324706FF-7CD4-4822-824E-9DCAB8D4079B}" name="Table1" displayName="Table1" ref="A1:F38" totalsRowShown="0" headerRowDxfId="8" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5">
   <autoFilter ref="A1:F38" xr:uid="{324706FF-7CD4-4822-824E-9DCAB8D4079B}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{688B2420-8DD1-4212-B637-1E01C0566A63}" name="Code" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{9A8A1365-EEE0-4926-A2C8-49E7D41EFC20}" name="Species" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{E75B966B-CCEA-426B-9D86-367E364C1280}" name="Type" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{EE9CBF76-25C2-4091-90B1-092311E311B6}" name="Familia" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{A28F9AA2-4F35-4BFD-B350-88646FCEBC86}" name="Genero" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{688B2420-8DD1-4212-B637-1E01C0566A63}" name="Code" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{9A8A1365-EEE0-4926-A2C8-49E7D41EFC20}" name="Species" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{E75B966B-CCEA-426B-9D86-367E364C1280}" name="Type" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{EE9CBF76-25C2-4091-90B1-092311E311B6}" name="Familia" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{A28F9AA2-4F35-4BFD-B350-88646FCEBC86}" name="Genero" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{AC1CE9E6-0145-4A8B-A893-462A840F6F26}" name="Equation"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>

</xml_diff>